<commit_message>
Add dedicated unstake deep-dive test plan (37 cases)
- New csv/mexico_unstake_deep_dive.csv covering happy path, lock timing
  boundaries, IDOR/PDA spoofing, race conditions, atomicity/rent/compute
  budget, multisig pause behavior, rewards interaction (pending rewards,
  time-weighted tier accrual), and UI/UX for the unstake flow specifically
- Generalize build_master_workbook.py to read each checklist's own CSV
  columns (so the new Category column renders correctly) instead of a
  hardcoded 3-column schema
- Add the new checklist as an 'Unstake Deep Dive' tab in the master workbook
  and note the next priority action in the README

Co-authored-by: Mykola-Ursal <Mykola-Ursal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mexico-staking-qa/Mexico_Staking_QA_Master.xlsx
+++ b/mexico-staking-qa/Mexico_Staking_QA_Master.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Smoke Fast" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Break It Tonight" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Solana Specific" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Unstake Deep Dive" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -592,75 +593,126 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Unstake Deep Dive</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>37</v>
+      </c>
+      <c r="C7">
+        <f>COUNTIF('Unstake Deep Dive'!F2:F38,"Not tested")</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>COUNTIF('Unstake Deep Dive'!F2:F38,"Passed")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>COUNTIF('Unstake Deep Dive'!F2:F38,"Failed")</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>COUNTIF('Unstake Deep Dive'!F2:F38,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>COUNTIF('Unstake Deep Dive'!F2:F38,"Skipped")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B8" s="2">
-        <f>SUM(B4:B6)</f>
+      <c r="B9" s="2">
+        <f>SUM(B4:B7)</f>
         <v/>
       </c>
-      <c r="C8" s="2">
-        <f>SUM(C4:C6)</f>
+      <c r="C9" s="2">
+        <f>SUM(C4:C7)</f>
         <v/>
       </c>
-      <c r="D8" s="2">
-        <f>SUM(D4:D6)</f>
+      <c r="D9" s="2">
+        <f>SUM(D4:D7)</f>
         <v/>
       </c>
-      <c r="E8" s="2">
-        <f>SUM(E4:E6)</f>
+      <c r="E9" s="2">
+        <f>SUM(E4:E7)</f>
         <v/>
       </c>
-      <c r="F8" s="2">
-        <f>SUM(F4:F6)</f>
+      <c r="F9" s="2">
+        <f>SUM(F4:F7)</f>
         <v/>
       </c>
-      <c r="G8" s="2">
-        <f>SUM(G4:G6)</f>
+      <c r="G9" s="2">
+        <f>SUM(G4:G7)</f>
         <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Open findings not part of the original checklists (see bug_reports/):</t>
-        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BUG-001</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Helius RPC API key exposed in plain text query parameter on the front end</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Critical</t>
+          <t>Open findings not part of the original checklists (see bug_reports/):</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>BUG-001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Helius RPC API key exposed in plain text query parameter on the front end</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>BUG-002</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Verify rounding behavior on small/frequent claims (dust)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Medium — pending verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Note: 'Unstake Deep Dive' overlaps with unstake-related cases already present in the</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>other three checklists; treat it as the authoritative, expanded source for unstake and</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>avoid double-counting duplicate cases when tallying overall coverage.</t>
         </is>
       </c>
     </row>
@@ -679,11 +731,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1391,11 +1443,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2181,11 +2233,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2855,4 +2907,1219 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>How to test</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Full unstake immediately after unlock</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Happy path</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Wait until the position's lock-end timestamp passes, open the position, click "Unstake", approve in Phantom</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Transaction confirms</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Full unstake well after unlock (delayed, not immediate)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Happy path</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Let an unlocked position sit unclaimed/un-unstaked for a while, then unstake it</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Unstake still succeeds and pays out the correct amount per the reward spec (verify whether rewards keep accruing past unlock or freeze at unlock — behavior must match design, not just "seems fine")</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Sequential unstake of multiple independent positions</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Happy path</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Create 3+ independent positions from one wallet, unstake them one after another (A, then B, then C)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Each unstake is independent</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Unstake right at the unlock boundary (script/rapid retry near the exact timestamp)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Timing / lock</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Attempt unstake at, just before, and just after the on-chain unlock timestamp (e.g. loop-retry near the boundary)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Unstake is rejected strictly before the unlock timestamp and accepted at/after it — no off-by-one gap or premature acceptance</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Attempt unstake 1 second before unlock</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Timing / lock</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>With a position whose lock is about to end, attempt unstake slightly early</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Action is blocked by the UI and rejected on-chain if attempted directly</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Lock countdown shown in UI matches on-chain unlock timestamp</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Timing / lock</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Compare the UI's displayed "unlocks in ..." countdown against the on-chain lock-end value read directly from the position account</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Values match</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Device clock manipulation does not affect lock/unlock state</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Timing / lock</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Change the local device clock forward or backward by several days, then check the lock/unlock state and try to unstake</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>State and enforcement are based on on-chain Clock, not the device's system time — changing the device clock has no effect</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Attempt to unstake an already-closed/fully-unstaked position</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Fully unstake a position, then try to trigger "Unstake" on it again (e.g. via a stale UI tab, browser back button, or resubmitting the same request)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Clear error is shown ("position not found"/"already closed")</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Attempt unstake with insufficient SOL for the network fee</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Drain the wallet's SOL down to (near) zero, keep MEX staked, attempt unstake</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Transaction fails gracefully with an insufficient-funds-for-fee style error</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Attempt unstake while wallet session/connection is lost mid-flow</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Disconnect/lock Phantom after opening the unstake confirmation dialog but before signing, then try to proceed</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>UI prompts to reconnect</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Confirm whether partial unstake is supported, and test accordingly</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Check PRD/spec and UI for a partial-unstake option</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> if present, unstake less than the full staked amount and verify the remainder stays staked correctly</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Submit unstake instruction for a position PDA owned by another wallet (IDOR)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Security / IDOR</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Copy an unstake request from the Network tab, replace the position account with another (victim) wallet's known position PDA, sign as the attacker, submit directly</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Program rejects the instruction (signer is not the authority/owner on that position account)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Redirect unstake payout to an attacker-controlled destination account</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Security / IDOR</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Modify the intercepted unstake transaction's destination token account to an ATA that does not belong to the position's owner, then submit</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Program validates the destination account against the owner's associated token account and rejects the mismatched destination</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Bypass the UI's locked/disabled unstake button via a raw instruction</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Security / IDOR</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>While a position is still inside its lock window, copy the unstake request structure from Network tab and submit it directly (bypassing the disabled UI control)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Program rejects the unstake based on the on-chain lock-end check, independent of what the UI would allow to be built</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Pass a manually-derived, wrong-seed PDA as the position account</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Security / IDOR</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Craft an unstake instruction referencing a PDA that is syntactically valid but not derived from the correct seeds/bump for that position, submit it</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Program's account validation rejects the mismatched PDA</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Replay a previously confirmed unstake transaction</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Security / IDOR</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Resubmit the exact same fully-signed unstake transaction (same signature, same blockhash) after it has already been confirmed</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Second submission is rejected as already processed</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Attempt unstake using a stale/expired blockhash</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Security / IDOR</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Build and sign an unstake transaction, wait past the blockhash validity window (~60-90s), then submit</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Submission fails due to expired/not-found blockhash rather than executing with stale context</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Race two unstake requests on the same position</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Race condition</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Trigger "Unstake" on the same position twice in quick succession (two browser tabs or a rapid double-click bypassing any UI debounce)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Only the first request succeeds</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Race unstake and claim on the same position</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Race condition</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Simultaneously trigger "Unstake" and "Claim" on the same position (two tabs, near-simultaneous submission)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Requests resolve consistently — rewards are neither paid out twice nor silently lost between the two operations</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Race unstake and check-in at the moment of unlock</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Race condition</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>At the exact moment a position unlocks, simultaneously attempt a check-in and an unstake</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Both resolve in a well-defined, consistent order per the on-chain logic</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Atomicity when unstake bundles auto-compound-at-unlock in the same transaction</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Solana mechanics</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Force a failure partway through a combined unstake+auto-compound transaction (e.g. insufficient rent for a newly required account) and observe the result</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>The entire transaction fails and rolls back as a unit</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Network fee is charged even when the unstake instruction is rejected</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Solana mechanics</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Attempt an unstake that is expected to be rejected on-chain (e.g. raw instruction sent before unlock), inspect the fee payer's SOL balance before/after</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Behavior is verified and documented: either the fee is charged despite instruction failure (typical for on-chain program errors) or the request fails at simulation before broadcast (no fee) — confirm which applies here and that it matches user-facing messaging</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Compute budget is sufficient for unstake with many pending reward computations</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Solana mechanics</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Let a position accrue rewards across many check-in/tier changes, then unstake it and inspect compute units consumed on a devnet explorer</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Transaction confirms without exceeding the compute unit limit, or the app explicitly requests additional compute budget via `ComputeBudgetProgram` and still stays within protocol limits</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Position PDA account is closed and rent refunded on full unstake</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Rent / accounts</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Fully unstake a position and inspect the position PDA's account status and the recipient's SOL balance change on a devnet explorer</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>The position account is closed</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Wallet's MEX associated token account is not closed by unstake</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Rent / accounts</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Unstake a position fully, then check whether the wallet's MEX ATA still exists and is reusable</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>The ATA persists after unstake (only the position account should close) so future stakes don't need to re-pay ATA rent</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Closing one position's account does not affect sibling positions</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Rent / accounts</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>With 2+ independent positions open, fully unstake one of them and check the others</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>The remaining positions' balances, lock timers, and accounts are completely unaffected</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Unstake behavior when the pool/program is paused by admin multisig (if a pause mechanism exists)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Multisig / admin</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>If a Squads-controlled pause exists, have the multisig pause the program, then attempt to unstake a position</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Unstake is either explicitly blocked with a clear error (if pause covers withdrawals) or explicitly still allowed (if pause only affects new stakes) — confirm which is the intended behavior and that it's enforced on-chain, not just in the UI</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Unstake resumes correctly after an admin multisig unpause (if applicable)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Multisig / admin</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>After confirming pause blocks unstake (previous case), have the multisig execute an unpause action, then retry the same unstake</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Previously blocked unstake now succeeds without requiring the user to do anything beyond retrying</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Unstake a position with pending unclaimed rewards</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Rewards interaction</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Let rewards accrue without claiming, then unstake the position directly (without a separate claim first)</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Pending rewards are auto-settled per design (claimed/compounded as part of unstake) — verify they are not silently forfeited</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Unstake a position with zero pending rewards (already fully claimed)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Rewards interaction</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Claim all pending rewards on a position, then immediately unstake it</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Only the principal is returned</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Final payout reflects time-weighted tier progression, not a retroactive final tier</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Rewards interaction</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Progress a position through multiple check-in tiers over time (primary/secondary rate changes), then unstake and compare the total payout to a manual calculation based on the time actually spent at each tier</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Reward calculation uses the tier rate that was active during each accrual period, not the tier reached at the moment of unstake</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Unstake confirmation dialog shows an accurate principal/reward breakdown before signing</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Open the unstake confirmation modal for a position with known principal and accrued rewards</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Displayed amounts (principal, rewards, total) match what is actually transferred once the transaction confirms</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Rejecting the wallet signature popup during unstake leaves a clean state</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Start an unstake flow, but click "Reject" in the Phantom signature popup instead of approving</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>UI returns cleanly to the pre-unstake state</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Unstake button state matches fresh on-chain data after a hard reload</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Reload the page (hard refresh, clearing any client cache) right at/near a position's unlock boundary and check the unstake control's enabled/disabled state</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>State is derived from a fresh on-chain query and matches reality, not a stale cached client-side timer</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Position list updates immediately after a successful unstake</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Complete an unstake and observe the "My Positions" list without manually refreshing the page</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>The unstaked position disappears (or is marked closed) immediately after transaction confirmation</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Wallet balance updates immediately after a successful unstake</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Complete an unstake and observe the displayed MEX balance without manually refreshing the page</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>The balance reflects the newly returned principal/rewards immediately after confirmation</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Clear error is shown for non-lock-related unstake failures</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Simulate or trigger a non-lock unstake failure (e.g. network congestion, RPC timeout, simulation failure) and observe the UI's response</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>A clear, specific error message is shown to the user</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Passed,Failed,Blocked,Skipped"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2 G3 G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"P0,P1,P2,P3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>